<commit_message>
MAJ de FrPractitionerDocument+Ajout de ValueSets f67d951e8c9ee06bd10baad46d5f78256793e8fa
</commit_message>
<xml_diff>
--- a/htr-FHIR/ig/StructureDefinition-fr-location-document.xlsx
+++ b/htr-FHIR/ig/StructureDefinition-fr-location-document.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-03-25T14:07:20+00:00</t>
+    <t>2025-03-31T09:17:15+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -944,7 +944,7 @@
     <t>Location.type.coding</t>
   </si>
   <si>
-    <t xml:space="preserve"> Structure de prise en charge : healthCareFacility</t>
+    <t>Structure de prise en charge : healthCareFacility</t>
   </si>
   <si>
     <t>A reference to a code defined by a terminology system.</t>

</xml_diff>

<commit_message>
Update des profils FrComposition+FrLocationDocument 77807a3eb9ea2e58f8bd981383343550a916f47f
</commit_message>
<xml_diff>
--- a/htr-FHIR/ig/StructureDefinition-fr-location-document.xlsx
+++ b/htr-FHIR/ig/StructureDefinition-fr-location-document.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-06T15:53:54+00:00</t>
+    <t>2025-05-06T15:58:22+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -944,7 +944,7 @@
     <t>Location.type.coding</t>
   </si>
   <si>
-    <t>Structure de prise en charge : healthcareFacility</t>
+    <t>Structure de prise en charge : healthCareFacility</t>
   </si>
   <si>
     <t>A reference to a code defined by a terminology system.</t>

</xml_diff>